<commit_message>
Autofill new requests, team view, temperature 0, demo sets and leadership docs
- Requester form: prefill fields from uploaded documents (prefill.py, prefill.js)
- Buyer team view (team.py, team_routes, team.html)
- LLM calls now run at temperature 0
- Regenerated demo sets; removed old generated RFQ rounds and repository files
- Docs: leadership Q&A, business guide, demo script, technical guide, jury deck

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo_documents/portal_upload/CASE-31_Network_printers_branches/05_Quotation_Inkpoint.xlsx
+++ b/demo_documents/portal_upload/CASE-31_Network_printers_branches/05_Quotation_Inkpoint.xlsx
@@ -503,14 +503,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HP 151A Toner (W1510A)</t>
+          <t>APC BX1100C-IN UPS 1100VA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>6990</v>
+        <v>6280</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>83880</v>
+        <v>37680</v>
       </c>
     </row>
     <row r="9">
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>323880</v>
+        <v>277680</v>
       </c>
     </row>
     <row r="12">
@@ -635,7 +635,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HP 151A Toner (W1510A): Rs 6,990 per unit x 12</t>
+          <t>APC BX1100C-IN UPS 1100VA: Rs 6,280 per unit x 6</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Total Rs 3,23,880 exclusive of 18% GST.</t>
+          <t>Total Rs 2,77,680 exclusive of 18% GST.</t>
         </is>
       </c>
     </row>

</xml_diff>